<commit_message>
docs(AOFP-202): add report 5 test documentation and review 2 PDFs
</commit_message>
<xml_diff>
--- a/docs/review-2/source/Report3_Project_Tracking.xlsx
+++ b/docs/review-2/source/Report3_Project_Tracking.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12300" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12300" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q&amp;A" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$7:$G$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$B$3:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$7:$G$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$B$3:$I$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="35">
+  <fonts count="34">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -259,12 +259,6 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="36">
     <fill>
@@ -601,7 +595,7 @@
     </border>
   </borders>
   <cellStyleXfs count="51">
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0"/>
@@ -736,11 +730,10 @@
     <xf numFmtId="0" fontId="32" fillId="35" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -801,6 +794,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="51">
@@ -1369,1109 +1368,1112 @@
   <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.8285714285714" defaultRowHeight="14.25"/>
   <cols>
-    <col width="4.82857142857143" customWidth="1" style="14" min="1" max="1"/>
-    <col width="41.1619047619048" customWidth="1" style="15" min="2" max="2"/>
-    <col width="13.1142857142857" customWidth="1" style="15" min="3" max="3"/>
-    <col width="8.81904761904762" customWidth="1" style="15" min="4" max="4"/>
-    <col width="66.6666666666667" customWidth="1" style="15" min="5" max="5"/>
-    <col width="10.6571428571429" customWidth="1" style="15" min="6" max="6"/>
-    <col width="8.828571428571429" customWidth="1" style="15" min="7" max="228"/>
-    <col width="10.8285714285714" customWidth="1" style="15" min="229" max="16384"/>
+    <col width="4.82857142857143" customWidth="1" style="13" min="1" max="1"/>
+    <col width="41.1619047619048" customWidth="1" style="14" min="2" max="2"/>
+    <col width="13.1142857142857" customWidth="1" style="14" min="3" max="3"/>
+    <col width="8.81904761904762" customWidth="1" style="14" min="4" max="4"/>
+    <col width="66.6666666666667" customWidth="1" style="14" min="5" max="5"/>
+    <col width="10.6571428571429" customWidth="1" style="14" min="6" max="6"/>
+    <col width="8.828571428571429" customWidth="1" style="14" min="7" max="228"/>
+    <col width="10.8285714285714" customWidth="1" style="14" min="229" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.5" customHeight="1" s="1">
-      <c r="C1" s="14" t="n"/>
-    </row>
-    <row r="2" ht="13.5" customHeight="1" s="1">
-      <c r="C2" s="14" t="n"/>
-    </row>
-    <row r="3" ht="13.5" customHeight="1" s="1">
-      <c r="C3" s="14" t="n"/>
-    </row>
-    <row r="4" ht="13.5" customHeight="1" s="1">
-      <c r="C4" s="14" t="n"/>
-    </row>
-    <row r="5" ht="18.75" customHeight="1" s="1">
-      <c r="D5" s="16" t="inlineStr">
+    <row r="1" ht="13.5" customHeight="1">
+      <c r="C1" s="13" t="n"/>
+    </row>
+    <row r="2" ht="13.5" customHeight="1">
+      <c r="C2" s="13" t="n"/>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="C3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="13.5" customHeight="1">
+      <c r="C4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>PROJECT WORK BREAKDOWN STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="1">
-      <c r="A6" s="17" t="n"/>
-      <c r="C6" s="14" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="1">
-      <c r="A7" s="18" t="inlineStr">
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="16" t="n"/>
+      <c r="C6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Function/Screen</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Level*</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Function/Screen Details</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="41" customHeight="1" s="1">
-      <c r="A8" s="19">
+    <row r="8" ht="41" customHeight="1">
+      <c r="A8" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Login (e-mail, Google, two-factor)</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="31.5" customHeight="1" s="1">
-      <c r="A9" s="19">
+    <row r="9" ht="31.5" customHeight="1">
+      <c r="A9" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Forgot / Reset Password</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="31.5" customHeight="1" s="1">
-      <c r="A10" s="19">
+    <row r="10" ht="31.5" customHeight="1">
+      <c r="A10" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Change Password</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="31.5" customHeight="1" s="1">
-      <c r="A11" s="19">
+    <row r="11" ht="31.5" customHeight="1">
+      <c r="A11" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Profile &amp; Settings</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth + users</t>
         </is>
       </c>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="31.5" customHeight="1" s="1">
-      <c r="A12" s="19">
+    <row r="12" ht="31.5" customHeight="1">
+      <c r="A12" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Notifications</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: notifications</t>
         </is>
       </c>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="31.5" customHeight="1" s="1">
-      <c r="A13" s="19">
+    <row r="13" ht="31.5" customHeight="1">
+      <c r="A13" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Action History</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: history</t>
         </is>
       </c>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="31.5" customHeight="1" s="1">
-      <c r="A14" s="19">
+    <row r="14" ht="31.5" customHeight="1">
+      <c r="A14" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Dashboard Overview</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Packing report + packaging-savings APIs (modules packing, packaging-materials); revenue-by-channel, finance and staff widgets still use sample data (no back-end aggregate API)</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>Iteration 3</t>
         </is>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="31.5" customHeight="1" s="1">
-      <c r="A15" s="19">
+    <row r="15" ht="31.5" customHeight="1">
+      <c r="A15" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Omnichannel Orders / Order Detail</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: orders</t>
         </is>
       </c>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="31.5" customHeight="1" s="1">
-      <c r="A16" s="19">
+    <row r="16" ht="31.5" customHeight="1">
+      <c r="A16" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Groups &amp; Express</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: order-groups</t>
         </is>
       </c>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="31.5" customHeight="1" s="1">
-      <c r="A17" s="19">
+    <row r="17" ht="31.5" customHeight="1">
+      <c r="A17" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Order Sync Settings</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Simple</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>About 3 API endpoints of module: order-sync-settings</t>
         </is>
       </c>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="31.5" customHeight="1" s="1">
-      <c r="A18" s="19">
+    <row r="18" ht="31.5" customHeight="1">
+      <c r="A18" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Marketplace Connections</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: marketplace-integration</t>
         </is>
       </c>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="31.5" customHeight="1" s="1">
-      <c r="A19" s="19">
+    <row r="19" ht="31.5" customHeight="1">
+      <c r="A19" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Warehouse Picking</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: order-groups (picking part)</t>
         </is>
       </c>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="31.5" customHeight="1" s="1">
-      <c r="A20" s="19">
+    <row r="20" ht="31.5" customHeight="1">
+      <c r="A20" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Warehouse Inventory</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>About 39 API endpoints of module: warehouse</t>
         </is>
       </c>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="43" customHeight="1" s="1">
-      <c r="A21" s="19">
+    <row r="21" ht="43" customHeight="1">
+      <c r="A21" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Admin Warehouse (structure, SKUs, mappings)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>About 64 API endpoints of module: master-skus + categories + warehouse</t>
         </is>
       </c>
-      <c r="F21" s="20" t="n"/>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="31.5" customHeight="1" s="1">
-      <c r="A22" s="19">
+    <row r="22" ht="31.5" customHeight="1">
+      <c r="A22" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Product Master (packaging profile)</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>About 5 API endpoints of module: product-master</t>
         </is>
       </c>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="inlineStr">
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="31.5" customHeight="1" s="1">
-      <c r="A23" s="19">
+    <row r="23" ht="31.5" customHeight="1">
+      <c r="A23" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Packing Station</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>About 29 API endpoints of module: packing-plan</t>
         </is>
       </c>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="20" t="inlineStr">
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="31.5" customHeight="1" s="1">
-      <c r="A24" s="19">
+    <row r="24" ht="31.5" customHeight="1">
+      <c r="A24" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Admin Packing Plans</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>About 29 API endpoints of module: packing-plan</t>
         </is>
       </c>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="inlineStr">
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="31.5" customHeight="1" s="1">
-      <c r="A25" s="19">
+    <row r="25" ht="31.5" customHeight="1">
+      <c r="A25" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Packaging Rules / Materials</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>About 26 API endpoints of module: packaging-materials + packaging</t>
         </is>
       </c>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="inlineStr">
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="31.5" customHeight="1" s="1">
-      <c r="A26" s="19">
+    <row r="26" ht="31.5" customHeight="1">
+      <c r="A26" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Shipping &amp; Fulfillment</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>About 27 API endpoints of module: shipments + shipping</t>
         </is>
       </c>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="20" t="inlineStr">
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="31.5" customHeight="1" s="1">
-      <c r="A27" s="19">
+    <row r="27" ht="31.5" customHeight="1">
+      <c r="A27" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>About 12 API endpoints of module: returns</t>
         </is>
       </c>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="20" t="inlineStr">
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="31.5" customHeight="1" s="1">
-      <c r="A28" s="19">
+    <row r="28" ht="31.5" customHeight="1">
+      <c r="A28" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Staff Directory / Admin Roles</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>About 12 API endpoints of module: users + staff-assignment</t>
         </is>
       </c>
-      <c r="F28" s="20" t="n"/>
-      <c r="G28" s="20" t="inlineStr">
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="31.5" customHeight="1" s="1">
-      <c r="A29" s="19">
+    <row r="29" ht="31.5" customHeight="1">
+      <c r="A29" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>AURELLE Home / Shop / Product Detail</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F29" s="20" t="n"/>
-      <c r="G29" s="20" t="inlineStr">
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="31.5" customHeight="1" s="1">
-      <c r="A30" s="19">
+    <row r="30" ht="31.5" customHeight="1">
+      <c r="A30" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>AURELLE Cart / Checkout</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F30" s="20" t="n"/>
-      <c r="G30" s="20" t="inlineStr">
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="31.5" customHeight="1" s="1">
-      <c r="A31" s="19">
+    <row r="31" ht="31.5" customHeight="1">
+      <c r="A31" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>AURELLE My Orders / Order Detail</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F31" s="20" t="n"/>
-      <c r="G31" s="20" t="inlineStr">
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="31.5" customHeight="1" s="1">
-      <c r="A32" s="19">
+    <row r="32" ht="31.5" customHeight="1">
+      <c r="A32" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>AURELLE My Returns / Return Detail</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F32" s="20" t="n"/>
-      <c r="G32" s="20" t="inlineStr">
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="31.5" customHeight="1" s="1">
-      <c r="A33" s="19">
+    <row r="33" ht="31.5" customHeight="1">
+      <c r="A33" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>AURELLE Customer Login / Register</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: storefront customer-auth</t>
         </is>
       </c>
-      <c r="F33" s="20" t="n"/>
-      <c r="G33" s="20" t="inlineStr">
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="31.5" customHeight="1" s="1">
-      <c r="A34" s="19">
+    <row r="34" ht="31.5" customHeight="1">
+      <c r="A34" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>AURELLE Web Admin (Products, Categories)</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E34" s="11" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: storefront-admin</t>
         </is>
       </c>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="inlineStr">
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="31.5" customHeight="1" s="1">
-      <c r="A35" s="19">
+    <row r="35" ht="31.5" customHeight="1">
+      <c r="A35" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>AURELLE Developer Portal</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>Simple</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>About 3 API endpoints of module: storefront-admin-auth / developer</t>
         </is>
       </c>
-      <c r="F35" s="20" t="n"/>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="31.5" customHeight="1" s="1">
-      <c r="A36" s="19">
+    <row r="36" ht="31.5" customHeight="1">
+      <c r="A36" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Mobile App (picking / packing scan, shipment tracking, push notifications)</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>Not implemented in this release; scanning is done on the web portal (Warehouse Picking, Packing Station). Planned Flutter app, Report 2 WBS 4.2</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F36" s="19" t="inlineStr">
         <is>
           <t>Iteration 3</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="13.5" customHeight="1" s="1">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>(*) You can rate the functions' complexity based on the number of fields on the screens or the number of transactions in the function, with the details as below</t>
         </is>
       </c>
-      <c r="B37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-    </row>
-    <row r="38" ht="13.5" customHeight="1" s="1">
-      <c r="B38" s="23" t="inlineStr">
+      <c r="B37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>simple</t>
         </is>
       </c>
-      <c r="C38" s="24" t="inlineStr">
+      <c r="C38" s="23" t="inlineStr">
         <is>
           <t>&lt;=7 fields</t>
         </is>
       </c>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="24" t="inlineStr">
         <is>
           <t>&lt;=3 transactions</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="13.5" customHeight="1" s="1">
-      <c r="B39" s="23" t="inlineStr">
+    <row r="39" ht="13.5" customHeight="1">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="C39" s="23" t="inlineStr">
         <is>
           <t>&lt;=15 fields</t>
         </is>
       </c>
-      <c r="D39" s="25" t="inlineStr">
+      <c r="D39" s="24" t="inlineStr">
         <is>
           <t>&lt;= 7 transactions</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="13.5" customHeight="1" s="1">
-      <c r="B40" s="23" t="inlineStr">
+    <row r="40" ht="13.5" customHeight="1">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>complex</t>
         </is>
       </c>
-      <c r="C40" s="24" t="inlineStr">
+      <c r="C40" s="23" t="inlineStr">
         <is>
           <t>&gt;15 fields</t>
         </is>
       </c>
-      <c r="D40" s="25" t="inlineStr">
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>&gt; 7 transactions</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="13.5" customHeight="1" s="1">
-      <c r="A41" s="26" t="inlineStr">
+    <row r="41" ht="13.5" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>In which:</t>
         </is>
       </c>
-      <c r="B41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-    </row>
-    <row r="42" ht="13.5" customHeight="1" s="1">
-      <c r="A42" s="27" t="inlineStr">
+      <c r="B41" s="21" t="n"/>
+      <c r="D41" s="21" t="n"/>
+    </row>
+    <row r="42" ht="13.5" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
         <is>
           <t>fields: screen components or database table fields</t>
         </is>
       </c>
-      <c r="B42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
+      <c r="B42" s="21" t="n"/>
+      <c r="D42" s="21" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>transactions: action buttons, user or database transactions</t>
         </is>
       </c>
-      <c r="B43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-    </row>
-    <row r="44" ht="13.5" customHeight="1" s="1"/>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="B43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+    </row>
+    <row r="44" ht="13.5" customHeight="1"/>
+    <row r="45" ht="48" customHeight="1">
+      <c r="A45" s="28" t="inlineStr">
         <is>
           <t>Note: Level is estimated from the number of API endpoints (transactions) of the module behind each screen, so screens that share a large module appear as Complex. Status 'Done' = implemented in the repository, 'Doing' = partly implemented, 'Pending' = not started; Planned (iteration) is filled only for unfinished items.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:G42"/>
+  <autoFilter ref="A7:G43"/>
+  <mergeCells count="1">
+    <mergeCell ref="A45:G45"/>
+  </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D8:D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Simple,Medium,Complex"</formula1>
@@ -2495,313 +2497,409 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.5047619047619" defaultRowHeight="12.75"/>
   <cols>
-    <col width="4.16190476190476" customWidth="1" style="8" min="1" max="1"/>
-    <col width="30.3333333333333" customWidth="1" style="1" min="2" max="2"/>
-    <col width="34.8285714285714" customWidth="1" style="1" min="3" max="3"/>
-    <col width="11" customWidth="1" style="1" min="4" max="4"/>
-    <col width="10.6571428571429" customWidth="1" style="1" min="5" max="5"/>
-    <col width="12.1619047619048" customWidth="1" style="1" min="6" max="6"/>
-    <col width="12.5047619047619" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8.828571428571429" customWidth="1" style="1" min="8" max="8"/>
-    <col width="38.3333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="4.16190476190476" customWidth="1" style="7" min="1" max="1"/>
+    <col width="30.3333333333333" customWidth="1" min="2" max="2"/>
+    <col width="34.8285714285714" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10.6571428571429" customWidth="1" min="5" max="5"/>
+    <col width="12.1619047619048" customWidth="1" min="6" max="6"/>
+    <col width="12.5047619047619" customWidth="1" min="7" max="7"/>
+    <col width="8.828571428571429" customWidth="1" min="8" max="8"/>
+    <col width="38.3333333333333" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>PROJECT ISSUES</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="7">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="6">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Potential Impact</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Open Date</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Close Date</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1" s="1">
-      <c r="A4" s="10">
+    <row r="4">
+      <c r="A4" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Tiki and TikTok Shop adapter files exist in the code but are not registered; shops of these platforms cannot be connected and their orders are not processed.</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Out of scope for this release (partner API access constraints, see BM03 #1).</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I4" s="12" t="n"/>
-    </row>
-    <row r="5" ht="48" customHeight="1" s="1">
-      <c r="A5" s="10">
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t>BM03 #1; Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Lazada is read-only: order status changes are not written back to Lazada (only AURELLE gets write-back).</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Lazada customers do not see OptiPack status changes.</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n"/>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I5" s="12" t="n"/>
-    </row>
-    <row r="6" ht="48" customHeight="1" s="1">
-      <c r="A6" s="10">
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>No staging environment is declared; only local, Docker Compose and Kubernetes manifests exist (docs/DEPLOYMENT.md).</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Review 2 requires demos on a declared staging environment.</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n"/>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="48" customHeight="1" s="1">
-      <c r="A7" s="10">
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief R1 / G3 – before the Review 2 demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Collection packaging_recommendations is listed in the schema but no longer used by the current packing flow.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Entity in ERD / database without active code; may be flagged by the self-review.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Thi</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I7" s="12" t="n"/>
-    </row>
-    <row r="8" ht="48" customHeight="1" s="1">
-      <c r="A8" s="10">
+      <c r="I7" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G5 – due 20/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Only GHN is integrated as a live carrier; other carriers are mock or manual.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Shipping depends on one carrier API.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I8" s="12" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="1">
-      <c r="A9" s="10">
+      <c r="I8" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Mobile app (registration 3.2, Report 1 FE-06) is not implemented; planned for Iteration 3.</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Picking and packing scanning is available only on the web portal.</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>Việt</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I9" s="12" t="n"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" s="1">
-      <c r="A10" s="10">
+      <c r="I9" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G1 – due 20/11/2026 (Iteration 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Home dashboard widgets (revenue by channel, finance, staff) use sample data; the back end has no aggregate API for them.</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Store Owner cannot rely on these widgets; real figures are in packing reports and action history.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I10" s="12" t="n"/>
+      <c r="I10" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G2 – due 20/11/2026</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Automated back-end tests use mocked database models; there is no end-to-end test against a real MongoDB replica set.</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Transaction and index behaviour is not verified automatically end to end.</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>Thi</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I11" s="12" t="n"/>
+      <c r="I11" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G4 – due 04/12/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:I10"/>
+  <autoFilter ref="B3:I11"/>
   <dataValidations count="2">
     <dataValidation sqref="D4:D11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Low,Medium,High"</formula1>
@@ -2824,210 +2922,210 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.5047619047619" defaultRowHeight="12.75"/>
   <cols>
-    <col width="17.5047619047619" customWidth="1" style="1" min="2" max="2"/>
-    <col width="41.5047619047619" customWidth="1" style="1" min="4" max="4"/>
-    <col width="48.3333333333333" customWidth="1" style="1" min="7" max="7"/>
+    <col width="17.5047619047619" customWidth="1" min="2" max="2"/>
+    <col width="41.5047619047619" customWidth="1" min="4" max="4"/>
+    <col width="48.3333333333333" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PROJECT DEFECTS</t>
         </is>
       </c>
     </row>
-    <row r="3" s="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Function/Screen</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Tester</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Defect Description</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Assign To</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="4" s="1">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n"/>
-    </row>
-    <row r="5" s="1">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
-    </row>
-    <row r="6" s="1">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-    </row>
-    <row r="7" s="1">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-    </row>
-    <row r="8" s="1">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-    </row>
-    <row r="9" s="1">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-    </row>
-    <row r="10" s="1">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n"/>
-    </row>
-    <row r="11" s="1">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n"/>
-    </row>
-    <row r="12" s="1">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n"/>
-    </row>
-    <row r="13" s="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n"/>
-    </row>
-    <row r="14" s="1">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n"/>
-    </row>
-    <row r="15" s="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="G14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
+      <c r="G15" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3049,256 +3147,256 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.828571428571429" defaultRowHeight="12.75"/>
   <cols>
-    <col width="55" customWidth="1" style="1" min="2" max="2"/>
-    <col width="66.6666666666667" customWidth="1" style="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="66.6666666666667" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PROJECT Q&amp;A</t>
         </is>
       </c>
     </row>
-    <row r="3" s="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>By</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Note (answer, other notes)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="1">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="5" t="inlineStr">
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" s="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" s="1">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="F5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="1">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" s="1">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="F7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="1">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" s="1">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="F9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1" s="1">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="F10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" s="1">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="F11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1" s="1">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1" s="1">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="F13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1" s="1">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="15.75" customHeight="1" s="1">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="F15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
+      <c r="F16" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
docs(AOFP-219): sync guides storefront and reports from main
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/review-2/source/Report3_Project_Tracking.xlsx
+++ b/docs/review-2/source/Report3_Project_Tracking.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12300" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12300" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q&amp;A" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$7:$G$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$B$3:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$7:$G$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$B$3:$I$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="35">
+  <fonts count="34">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -259,12 +259,6 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="36">
     <fill>
@@ -601,7 +595,7 @@
     </border>
   </borders>
   <cellStyleXfs count="51">
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0"/>
@@ -736,11 +730,10 @@
     <xf numFmtId="0" fontId="32" fillId="35" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -801,6 +794,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="51">
@@ -1369,1109 +1368,1112 @@
   <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.8285714285714" defaultRowHeight="14.25"/>
   <cols>
-    <col width="4.82857142857143" customWidth="1" style="14" min="1" max="1"/>
-    <col width="41.1619047619048" customWidth="1" style="15" min="2" max="2"/>
-    <col width="13.1142857142857" customWidth="1" style="15" min="3" max="3"/>
-    <col width="8.81904761904762" customWidth="1" style="15" min="4" max="4"/>
-    <col width="66.6666666666667" customWidth="1" style="15" min="5" max="5"/>
-    <col width="10.6571428571429" customWidth="1" style="15" min="6" max="6"/>
-    <col width="8.828571428571429" customWidth="1" style="15" min="7" max="228"/>
-    <col width="10.8285714285714" customWidth="1" style="15" min="229" max="16384"/>
+    <col width="4.82857142857143" customWidth="1" style="13" min="1" max="1"/>
+    <col width="41.1619047619048" customWidth="1" style="14" min="2" max="2"/>
+    <col width="13.1142857142857" customWidth="1" style="14" min="3" max="3"/>
+    <col width="8.81904761904762" customWidth="1" style="14" min="4" max="4"/>
+    <col width="66.6666666666667" customWidth="1" style="14" min="5" max="5"/>
+    <col width="10.6571428571429" customWidth="1" style="14" min="6" max="6"/>
+    <col width="8.828571428571429" customWidth="1" style="14" min="7" max="228"/>
+    <col width="10.8285714285714" customWidth="1" style="14" min="229" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.5" customHeight="1" s="1">
-      <c r="C1" s="14" t="n"/>
-    </row>
-    <row r="2" ht="13.5" customHeight="1" s="1">
-      <c r="C2" s="14" t="n"/>
-    </row>
-    <row r="3" ht="13.5" customHeight="1" s="1">
-      <c r="C3" s="14" t="n"/>
-    </row>
-    <row r="4" ht="13.5" customHeight="1" s="1">
-      <c r="C4" s="14" t="n"/>
-    </row>
-    <row r="5" ht="18.75" customHeight="1" s="1">
-      <c r="D5" s="16" t="inlineStr">
+    <row r="1" ht="13.5" customHeight="1">
+      <c r="C1" s="13" t="n"/>
+    </row>
+    <row r="2" ht="13.5" customHeight="1">
+      <c r="C2" s="13" t="n"/>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="C3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="13.5" customHeight="1">
+      <c r="C4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>PROJECT WORK BREAKDOWN STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="1">
-      <c r="A6" s="17" t="n"/>
-      <c r="C6" s="14" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="1">
-      <c r="A7" s="18" t="inlineStr">
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="16" t="n"/>
+      <c r="C6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Function/Screen</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Level*</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Function/Screen Details</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="41" customHeight="1" s="1">
-      <c r="A8" s="19">
+    <row r="8" ht="41" customHeight="1">
+      <c r="A8" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Login (e-mail, Google, two-factor)</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="31.5" customHeight="1" s="1">
-      <c r="A9" s="19">
+    <row r="9" ht="31.5" customHeight="1">
+      <c r="A9" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Forgot / Reset Password</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="31.5" customHeight="1" s="1">
-      <c r="A10" s="19">
+    <row r="10" ht="31.5" customHeight="1">
+      <c r="A10" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Change Password</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth</t>
         </is>
       </c>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="31.5" customHeight="1" s="1">
-      <c r="A11" s="19">
+    <row r="11" ht="31.5" customHeight="1">
+      <c r="A11" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Profile &amp; Settings</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>About 10 API endpoints of module: auth + users</t>
         </is>
       </c>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="31.5" customHeight="1" s="1">
-      <c r="A12" s="19">
+    <row r="12" ht="31.5" customHeight="1">
+      <c r="A12" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Notifications</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: notifications</t>
         </is>
       </c>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="31.5" customHeight="1" s="1">
-      <c r="A13" s="19">
+    <row r="13" ht="31.5" customHeight="1">
+      <c r="A13" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Action History</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: history</t>
         </is>
       </c>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="31.5" customHeight="1" s="1">
-      <c r="A14" s="19">
+    <row r="14" ht="31.5" customHeight="1">
+      <c r="A14" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Dashboard Overview</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Packing report + packaging-savings APIs (modules packing, packaging-materials); revenue-by-channel, finance and staff widgets still use sample data (no back-end aggregate API)</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>Iteration 3</t>
         </is>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="31.5" customHeight="1" s="1">
-      <c r="A15" s="19">
+    <row r="15" ht="31.5" customHeight="1">
+      <c r="A15" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Omnichannel Orders / Order Detail</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: orders</t>
         </is>
       </c>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="31.5" customHeight="1" s="1">
-      <c r="A16" s="19">
+    <row r="16" ht="31.5" customHeight="1">
+      <c r="A16" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Groups &amp; Express</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: order-groups</t>
         </is>
       </c>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="31.5" customHeight="1" s="1">
-      <c r="A17" s="19">
+    <row r="17" ht="31.5" customHeight="1">
+      <c r="A17" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Order Sync Settings</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Simple</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>About 3 API endpoints of module: order-sync-settings</t>
         </is>
       </c>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="31.5" customHeight="1" s="1">
-      <c r="A18" s="19">
+    <row r="18" ht="31.5" customHeight="1">
+      <c r="A18" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Marketplace Connections</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: marketplace-integration</t>
         </is>
       </c>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="31.5" customHeight="1" s="1">
-      <c r="A19" s="19">
+    <row r="19" ht="31.5" customHeight="1">
+      <c r="A19" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Warehouse Picking</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: order-groups (picking part)</t>
         </is>
       </c>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="31.5" customHeight="1" s="1">
-      <c r="A20" s="19">
+    <row r="20" ht="31.5" customHeight="1">
+      <c r="A20" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Warehouse Inventory</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>About 39 API endpoints of module: warehouse</t>
         </is>
       </c>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="43" customHeight="1" s="1">
-      <c r="A21" s="19">
+    <row r="21" ht="43" customHeight="1">
+      <c r="A21" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Admin Warehouse (structure, SKUs, mappings)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>About 64 API endpoints of module: master-skus + categories + warehouse</t>
         </is>
       </c>
-      <c r="F21" s="20" t="n"/>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="31.5" customHeight="1" s="1">
-      <c r="A22" s="19">
+    <row r="22" ht="31.5" customHeight="1">
+      <c r="A22" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Product Master (packaging profile)</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>About 5 API endpoints of module: product-master</t>
         </is>
       </c>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="inlineStr">
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="31.5" customHeight="1" s="1">
-      <c r="A23" s="19">
+    <row r="23" ht="31.5" customHeight="1">
+      <c r="A23" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Packing Station</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>About 29 API endpoints of module: packing-plan</t>
         </is>
       </c>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="20" t="inlineStr">
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="31.5" customHeight="1" s="1">
-      <c r="A24" s="19">
+    <row r="24" ht="31.5" customHeight="1">
+      <c r="A24" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Admin Packing Plans</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>About 29 API endpoints of module: packing-plan</t>
         </is>
       </c>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="inlineStr">
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="31.5" customHeight="1" s="1">
-      <c r="A25" s="19">
+    <row r="25" ht="31.5" customHeight="1">
+      <c r="A25" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Packaging Rules / Materials</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>Packing</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>About 26 API endpoints of module: packaging-materials + packaging</t>
         </is>
       </c>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="inlineStr">
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="31.5" customHeight="1" s="1">
-      <c r="A26" s="19">
+    <row r="26" ht="31.5" customHeight="1">
+      <c r="A26" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Shipping &amp; Fulfillment</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>About 27 API endpoints of module: shipments + shipping</t>
         </is>
       </c>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="20" t="inlineStr">
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="31.5" customHeight="1" s="1">
-      <c r="A27" s="19">
+    <row r="27" ht="31.5" customHeight="1">
+      <c r="A27" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>About 12 API endpoints of module: returns</t>
         </is>
       </c>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="20" t="inlineStr">
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="31.5" customHeight="1" s="1">
-      <c r="A28" s="19">
+    <row r="28" ht="31.5" customHeight="1">
+      <c r="A28" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Staff Directory / Admin Roles</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>About 12 API endpoints of module: users + staff-assignment</t>
         </is>
       </c>
-      <c r="F28" s="20" t="n"/>
-      <c r="G28" s="20" t="inlineStr">
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="31.5" customHeight="1" s="1">
-      <c r="A29" s="19">
+    <row r="29" ht="31.5" customHeight="1">
+      <c r="A29" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>AURELLE Home / Shop / Product Detail</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F29" s="20" t="n"/>
-      <c r="G29" s="20" t="inlineStr">
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="31.5" customHeight="1" s="1">
-      <c r="A30" s="19">
+    <row r="30" ht="31.5" customHeight="1">
+      <c r="A30" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>AURELLE Cart / Checkout</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F30" s="20" t="n"/>
-      <c r="G30" s="20" t="inlineStr">
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="31.5" customHeight="1" s="1">
-      <c r="A31" s="19">
+    <row r="31" ht="31.5" customHeight="1">
+      <c r="A31" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>AURELLE My Orders / Order Detail</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F31" s="20" t="n"/>
-      <c r="G31" s="20" t="inlineStr">
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="31.5" customHeight="1" s="1">
-      <c r="A32" s="19">
+    <row r="32" ht="31.5" customHeight="1">
+      <c r="A32" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>AURELLE My Returns / Return Detail</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>About 19 API endpoints of module: storefront</t>
         </is>
       </c>
-      <c r="F32" s="20" t="n"/>
-      <c r="G32" s="20" t="inlineStr">
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="31.5" customHeight="1" s="1">
-      <c r="A33" s="19">
+    <row r="33" ht="31.5" customHeight="1">
+      <c r="A33" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>AURELLE Customer Login / Register</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>About 4 API endpoints of module: storefront customer-auth</t>
         </is>
       </c>
-      <c r="F33" s="20" t="n"/>
-      <c r="G33" s="20" t="inlineStr">
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="31.5" customHeight="1" s="1">
-      <c r="A34" s="19">
+    <row r="34" ht="31.5" customHeight="1">
+      <c r="A34" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>AURELLE Web Admin (Products, Categories)</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E34" s="11" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>About 15 API endpoints of module: storefront-admin</t>
         </is>
       </c>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="inlineStr">
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="31.5" customHeight="1" s="1">
-      <c r="A35" s="19">
+    <row r="35" ht="31.5" customHeight="1">
+      <c r="A35" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>AURELLE Developer Portal</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>AURELLE</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>Simple</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>About 3 API endpoints of module: storefront-admin-auth / developer</t>
         </is>
       </c>
-      <c r="F35" s="20" t="n"/>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="31.5" customHeight="1" s="1">
-      <c r="A36" s="19">
+    <row r="36" ht="31.5" customHeight="1">
+      <c r="A36" s="18">
         <f>ROW()-7</f>
         <v/>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Mobile App (picking / packing scan, shipment tracking, push notifications)</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>Complex</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>Not implemented in this release; scanning is done on the web portal (Warehouse Picking, Packing Station). Planned Flutter app, Report 2 WBS 4.2</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F36" s="19" t="inlineStr">
         <is>
           <t>Iteration 3</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="13.5" customHeight="1" s="1">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>(*) You can rate the functions' complexity based on the number of fields on the screens or the number of transactions in the function, with the details as below</t>
         </is>
       </c>
-      <c r="B37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-    </row>
-    <row r="38" ht="13.5" customHeight="1" s="1">
-      <c r="B38" s="23" t="inlineStr">
+      <c r="B37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>simple</t>
         </is>
       </c>
-      <c r="C38" s="24" t="inlineStr">
+      <c r="C38" s="23" t="inlineStr">
         <is>
           <t>&lt;=7 fields</t>
         </is>
       </c>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="24" t="inlineStr">
         <is>
           <t>&lt;=3 transactions</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="13.5" customHeight="1" s="1">
-      <c r="B39" s="23" t="inlineStr">
+    <row r="39" ht="13.5" customHeight="1">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="C39" s="23" t="inlineStr">
         <is>
           <t>&lt;=15 fields</t>
         </is>
       </c>
-      <c r="D39" s="25" t="inlineStr">
+      <c r="D39" s="24" t="inlineStr">
         <is>
           <t>&lt;= 7 transactions</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="13.5" customHeight="1" s="1">
-      <c r="B40" s="23" t="inlineStr">
+    <row r="40" ht="13.5" customHeight="1">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>complex</t>
         </is>
       </c>
-      <c r="C40" s="24" t="inlineStr">
+      <c r="C40" s="23" t="inlineStr">
         <is>
           <t>&gt;15 fields</t>
         </is>
       </c>
-      <c r="D40" s="25" t="inlineStr">
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>&gt; 7 transactions</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="13.5" customHeight="1" s="1">
-      <c r="A41" s="26" t="inlineStr">
+    <row r="41" ht="13.5" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>In which:</t>
         </is>
       </c>
-      <c r="B41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-    </row>
-    <row r="42" ht="13.5" customHeight="1" s="1">
-      <c r="A42" s="27" t="inlineStr">
+      <c r="B41" s="21" t="n"/>
+      <c r="D41" s="21" t="n"/>
+    </row>
+    <row r="42" ht="13.5" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
         <is>
           <t>fields: screen components or database table fields</t>
         </is>
       </c>
-      <c r="B42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
+      <c r="B42" s="21" t="n"/>
+      <c r="D42" s="21" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>transactions: action buttons, user or database transactions</t>
         </is>
       </c>
-      <c r="B43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-    </row>
-    <row r="44" ht="13.5" customHeight="1" s="1"/>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="B43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+    </row>
+    <row r="44" ht="13.5" customHeight="1"/>
+    <row r="45" ht="48" customHeight="1">
+      <c r="A45" s="28" t="inlineStr">
         <is>
           <t>Note: Level is estimated from the number of API endpoints (transactions) of the module behind each screen, so screens that share a large module appear as Complex. Status 'Done' = implemented in the repository, 'Doing' = partly implemented, 'Pending' = not started; Planned (iteration) is filled only for unfinished items.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:G42"/>
+  <autoFilter ref="A7:G43"/>
+  <mergeCells count="1">
+    <mergeCell ref="A45:G45"/>
+  </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D8:D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Simple,Medium,Complex"</formula1>
@@ -2495,313 +2497,409 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.5047619047619" defaultRowHeight="12.75"/>
   <cols>
-    <col width="4.16190476190476" customWidth="1" style="8" min="1" max="1"/>
-    <col width="30.3333333333333" customWidth="1" style="1" min="2" max="2"/>
-    <col width="34.8285714285714" customWidth="1" style="1" min="3" max="3"/>
-    <col width="11" customWidth="1" style="1" min="4" max="4"/>
-    <col width="10.6571428571429" customWidth="1" style="1" min="5" max="5"/>
-    <col width="12.1619047619048" customWidth="1" style="1" min="6" max="6"/>
-    <col width="12.5047619047619" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8.828571428571429" customWidth="1" style="1" min="8" max="8"/>
-    <col width="38.3333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="4.16190476190476" customWidth="1" style="7" min="1" max="1"/>
+    <col width="30.3333333333333" customWidth="1" min="2" max="2"/>
+    <col width="34.8285714285714" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10.6571428571429" customWidth="1" min="5" max="5"/>
+    <col width="12.1619047619048" customWidth="1" min="6" max="6"/>
+    <col width="12.5047619047619" customWidth="1" min="7" max="7"/>
+    <col width="8.828571428571429" customWidth="1" min="8" max="8"/>
+    <col width="38.3333333333333" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>PROJECT ISSUES</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="7">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="6">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Potential Impact</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Open Date</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Close Date</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1" s="1">
-      <c r="A4" s="10">
+    <row r="4">
+      <c r="A4" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Tiki and TikTok Shop adapter files exist in the code but are not registered; shops of these platforms cannot be connected and their orders are not processed.</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Out of scope for this release (partner API access constraints, see BM03 #1).</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I4" s="12" t="n"/>
-    </row>
-    <row r="5" ht="48" customHeight="1" s="1">
-      <c r="A5" s="10">
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t>BM03 #1; Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Lazada is read-only: order status changes are not written back to Lazada (only AURELLE gets write-back).</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Lazada customers do not see OptiPack status changes.</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n"/>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I5" s="12" t="n"/>
-    </row>
-    <row r="6" ht="48" customHeight="1" s="1">
-      <c r="A6" s="10">
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>No staging environment is declared; only local, Docker Compose and Kubernetes manifests exist (docs/DEPLOYMENT.md).</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Review 2 requires demos on a declared staging environment.</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n"/>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="48" customHeight="1" s="1">
-      <c r="A7" s="10">
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief R1 / G3 – before the Review 2 demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Collection packaging_recommendations is listed in the schema but no longer used by the current packing flow.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Entity in ERD / database without active code; may be flagged by the self-review.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Thi</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I7" s="12" t="n"/>
-    </row>
-    <row r="8" ht="48" customHeight="1" s="1">
-      <c r="A8" s="10">
+      <c r="I7" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G5 – due 20/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Only GHN is integrated as a live carrier; other carriers are mock or manual.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Shipping depends on one carrier API.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I8" s="12" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="1">
-      <c r="A9" s="10">
+      <c r="I8" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief 1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Mobile app (registration 3.2, Report 1 FE-06) is not implemented; planned for Iteration 3.</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Picking and packing scanning is available only on the web portal.</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>Việt</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I9" s="12" t="n"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" s="1">
-      <c r="A10" s="10">
+      <c r="I9" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G1 – due 20/11/2026 (Iteration 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Home dashboard widgets (revenue by channel, finance, staff) use sample data; the back end has no aggregate API for them.</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Store Owner cannot rely on these widgets; real figures are in packing reports and action history.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Thuận</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I10" s="12" t="n"/>
+      <c r="I10" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G2 – due 20/11/2026</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <f>ROW()-3</f>
         <v/>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Automated back-end tests use mocked database models; there is no end-to-end test against a real MongoDB replica set.</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Transaction and index behaviour is not verified automatically end to end.</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>Thi</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I11" s="12" t="n"/>
+      <c r="I11" s="27" t="inlineStr">
+        <is>
+          <t>Design Brief G4 – due 04/12/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:I10"/>
+  <autoFilter ref="B3:I11"/>
   <dataValidations count="2">
     <dataValidation sqref="D4:D11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Low,Medium,High"</formula1>
@@ -2824,210 +2922,210 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.5047619047619" defaultRowHeight="12.75"/>
   <cols>
-    <col width="17.5047619047619" customWidth="1" style="1" min="2" max="2"/>
-    <col width="41.5047619047619" customWidth="1" style="1" min="4" max="4"/>
-    <col width="48.3333333333333" customWidth="1" style="1" min="7" max="7"/>
+    <col width="17.5047619047619" customWidth="1" min="2" max="2"/>
+    <col width="41.5047619047619" customWidth="1" min="4" max="4"/>
+    <col width="48.3333333333333" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PROJECT DEFECTS</t>
         </is>
       </c>
     </row>
-    <row r="3" s="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Function/Screen</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Tester</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Defect Description</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Assign To</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="4" s="1">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n"/>
-    </row>
-    <row r="5" s="1">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
-    </row>
-    <row r="6" s="1">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-    </row>
-    <row r="7" s="1">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-    </row>
-    <row r="8" s="1">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-    </row>
-    <row r="9" s="1">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-    </row>
-    <row r="10" s="1">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n"/>
-    </row>
-    <row r="11" s="1">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n"/>
-    </row>
-    <row r="12" s="1">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n"/>
-    </row>
-    <row r="13" s="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n"/>
-    </row>
-    <row r="14" s="1">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n"/>
-    </row>
-    <row r="15" s="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="G14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
+      <c r="G15" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3049,256 +3147,256 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.828571428571429" defaultRowHeight="12.75"/>
   <cols>
-    <col width="55" customWidth="1" style="1" min="2" max="2"/>
-    <col width="66.6666666666667" customWidth="1" style="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="66.6666666666667" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PROJECT Q&amp;A</t>
         </is>
       </c>
     </row>
-    <row r="3" s="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>By</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Note (answer, other notes)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="1">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="5" t="inlineStr">
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" s="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" s="1">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="F5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="1">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" s="1">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="F7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="1">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" s="1">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="F9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1" s="1">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="F10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" s="1">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="F11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1" s="1">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1" s="1">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="F13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1" s="1">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="15.75" customHeight="1" s="1">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="F15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
+      <c r="F16" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>